<commit_message>
added restaurant customer survey results spreadsheet update
</commit_message>
<xml_diff>
--- a/week-01/The Simpson Restaurant & Bar.xlsx
+++ b/week-01/The Simpson Restaurant & Bar.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30610"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30610"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qinzen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="155" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BCCE43-6A9C-4AA8-8C97-F4E6F19068AF}"/>
+  <xr:revisionPtr revIDLastSave="256" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E434AE-63DC-47E7-8167-547B264EB43F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="forms_results" sheetId="1" r:id="rId1"/>
+    <sheet name="Pivot_Charts" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="98" r:id="rId3"/>
-    <pivotCache cacheId="113" r:id="rId4"/>
+    <pivotCache cacheId="79" r:id="rId3"/>
+    <pivotCache cacheId="83" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
   <si>
     <t>Id</t>
   </si>
@@ -172,33 +172,66 @@
     <t>Earning points towards free meals;Coupons or deals (BOGO);Members-only promotions;</t>
   </si>
   <si>
+    <t>dmendez1@my.yearupunited.org</t>
+  </si>
+  <si>
+    <t>denae mendez</t>
+  </si>
+  <si>
+    <t>Discounts on future purchases;Earning points towards free meals;Birthday Rewards</t>
+  </si>
+  <si>
+    <t>Frequent Visitors</t>
+  </si>
+  <si>
+    <t>Count of visitors</t>
+  </si>
+  <si>
+    <t>Restaurant Choice Reason</t>
+  </si>
+  <si>
+    <t>Number chosen</t>
+  </si>
+  <si>
+    <t>Promo Deal</t>
+  </si>
+  <si>
+    <t>How many chose</t>
+  </si>
+  <si>
     <t>Earning points towards free meals</t>
   </si>
   <si>
+    <t>Birthday Rewards</t>
+  </si>
+  <si>
+    <t>Several times a week</t>
+  </si>
+  <si>
     <t>Location</t>
   </si>
   <si>
-    <t>Birthday Rewards</t>
+    <t>Discounts</t>
+  </si>
+  <si>
+    <t>Monthly</t>
   </si>
   <si>
     <t>Atmosphere</t>
   </si>
   <si>
-    <t>Discounts</t>
+    <t>Coupons or Deals</t>
   </si>
   <si>
     <t>Grade</t>
   </si>
   <si>
-    <t>Coupons or Deals</t>
+    <t>Members-only promos</t>
   </si>
   <si>
     <t>Type of Restaurant/Cuisine (Italian, Greek, etc.)</t>
   </si>
   <si>
-    <t>Members-only promos</t>
-  </si>
-  <si>
     <t>Menu Options</t>
   </si>
   <si>
@@ -206,6 +239,9 @@
   </si>
   <si>
     <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of How many chose</t>
   </si>
 </sst>
 </file>
@@ -232,7 +268,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -240,139 +276,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="65"/>
-      </left>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="65"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="45" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,7 +373,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[The Simpson Restaurant &amp; Bar.xlsx]Sheet2!PivotTable1</c:name>
+    <c:name>[The Simpson Restaurant &amp; Bar.xlsx]Pivot_Charts!PivotTable1</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
@@ -585,7 +502,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet2!$B$2</c:f>
+              <c:f>Pivot_Charts!$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -606,9 +523,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet2!$A$3:$A$6</c:f>
+              <c:f>Pivot_Charts!$A$3:$A$7</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -618,15 +535,18 @@
                 <c:pt idx="2">
                   <c:v>5</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$B$3:$B$6</c:f>
+              <c:f>Pivot_Charts!$B$3:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -635,6 +555,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -926,6 +849,559 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[The Simpson Restaurant &amp; Bar.xlsx]Pivot_Charts!PivotTable2</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Preferred Promo Deal</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Pivot_Charts!$B$18</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Pivot_Charts!$A$19:$A$24</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Birthday Rewards</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Coupons or Deals</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Discounts</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Earning points towards free meals</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Members-only promos</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Pivot_Charts!$B$19:$B$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-202E-4188-91B2-56DDEB831AE7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="33"/>
+        <c:overlap val="-30"/>
+        <c:axId val="1969424392"/>
+        <c:axId val="11046919"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1969424392"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Promo Deal</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="11046919"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="11046919"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>How many chose</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1969424392"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -966,7 +1442,552 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1509,29 +2530,62 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>952500</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2" descr="Chart type: Clustered Bar. 'How many chose' by 'Promo Deal'&#10;&#10;Description automatically generated">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E3B1386-153E-C7F1-293A-F93F658376FD}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{E8587C62-DFE3-63A2-40ED-F951FCDEB51F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46311.628476041667" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="5" xr:uid="{314E3899-F73A-4104-87A1-DA6341D65789}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46312.464370949077" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{314E3899-F73A-4104-87A1-DA6341D65789}">
   <cacheSource type="worksheet">
     <worksheetSource name="OfficeForms.Table"/>
   </cacheSource>
   <cacheFields count="17">
     <cacheField name="Id" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5" count="5">
-        <n v="1"/>
-        <n v="2"/>
-        <n v="3"/>
-        <n v="4"/>
-        <n v="5"/>
-      </sharedItems>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="6"/>
     </cacheField>
     <cacheField name="Start time" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T20:52:24" maxDate="2026-10-16T11:13:50"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T20:52:24" maxDate="2026-10-16T16:32:30"/>
     </cacheField>
     <cacheField name="Completion time" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T20:55:37" maxDate="2026-10-16T11:15:12"/>
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-10-14T20:55:37" maxDate="2026-10-16T16:33:32"/>
     </cacheField>
     <cacheField name="Time to complete" numFmtId="45">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="1899-12-30T00:00:45" maxDate="1899-12-30T00:03:13"/>
@@ -1540,22 +2594,17 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="Name" numFmtId="0">
-      <sharedItems count="5">
-        <s v="gbolahan abidemi"/>
-        <s v="ardita mrapshtija"/>
-        <s v="idasha lee"/>
-        <s v="thania staana"/>
-        <s v="ajani lewis"/>
-      </sharedItems>
+      <sharedItems/>
     </cacheField>
     <cacheField name="How often do you visit us?" numFmtId="0">
       <sharedItems/>
     </cacheField>
     <cacheField name="How satisfied are you with your experience today?" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5" count="3">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="5" count="4">
         <n v="1"/>
         <n v="5"/>
         <n v="4"/>
+        <n v="3"/>
       </sharedItems>
     </cacheField>
     <cacheField name="How satisfied were you with the following?.Food quality" numFmtId="0">
@@ -1580,13 +2629,7 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="9"/>
     </cacheField>
     <cacheField name="Which Loyalty Program would interest you? (Pick up to 3)" numFmtId="0">
-      <sharedItems count="5">
-        <s v="None, this place STINKS;"/>
-        <s v="Earning points towards free meals;Discounts on future purchases;"/>
-        <s v="Birthday Rewards;Coupons or deals (BOGO);Discounts on future purchases;"/>
-        <s v="Members-only promotions;Coupons or deals (BOGO);Earning points towards free meals;"/>
-        <s v="Earning points towards free meals;Coupons or deals (BOGO);Members-only promotions;"/>
-      </sharedItems>
+      <sharedItems/>
     </cacheField>
     <cacheField name="Any feedback for us or anything we could do to improve your experience?" numFmtId="0">
       <sharedItems containsBlank="1"/>
@@ -1604,21 +2647,22 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46311.6426244213" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="4" xr:uid="{52B06EB2-1865-4668-BC48-C3D70E595F86}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46312.464370949077" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="5" xr:uid="{D43584F5-198D-4B50-B401-E83A77804DAE}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="O25:P29" sheet="Sheet1"/>
+    <worksheetSource ref="O24:P29" sheet="forms_results"/>
   </cacheSource>
   <cacheFields count="2">
-    <cacheField name="Earning points towards free meals" numFmtId="0">
-      <sharedItems count="4">
+    <cacheField name="Promo Deal" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Earning points towards free meals"/>
         <s v="Birthday Rewards"/>
         <s v="Discounts"/>
         <s v="Coupons or Deals"/>
         <s v="Members-only promos"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="3" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="3"/>
+    <cacheField name="How many chose" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2" maxValue="4"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1633,14 +2677,14 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="5">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="6">
   <r>
-    <x v="0"/>
+    <n v="1"/>
     <d v="2026-10-14T20:52:24"/>
     <d v="2026-10-14T20:55:37"/>
     <d v="1899-12-30T00:03:13"/>
     <s v="gabidemi@my.yearupunited.org"/>
-    <x v="0"/>
+    <s v="gbolahan abidemi"/>
     <s v="First visit"/>
     <x v="0"/>
     <s v="Dissatisfied"/>
@@ -1650,16 +2694,16 @@
     <s v="Very Dissatisfied"/>
     <s v="Pricing"/>
     <n v="1"/>
-    <x v="0"/>
+    <s v="None, this place STINKS;"/>
     <s v="Why were there flies hovering around my food!"/>
   </r>
   <r>
-    <x v="1"/>
+    <n v="2"/>
     <d v="2026-10-15T14:26:01"/>
     <d v="2026-10-15T14:26:46"/>
     <d v="1899-12-30T00:00:45"/>
     <s v="amrapshtija@my.yearupunited.org"/>
-    <x v="1"/>
+    <s v="ardita mrapshtija"/>
     <s v="Once a week"/>
     <x v="1"/>
     <s v="Dissatisfied"/>
@@ -1669,16 +2713,16 @@
     <s v="Neutral"/>
     <s v="Food Quality"/>
     <n v="4"/>
-    <x v="1"/>
+    <s v="Earning points towards free meals;Discounts on future purchases;"/>
     <m/>
   </r>
   <r>
-    <x v="2"/>
+    <n v="3"/>
     <d v="2026-10-15T14:45:13"/>
     <d v="2026-10-15T14:47:45"/>
     <d v="1899-12-30T00:02:32"/>
     <s v="ilee@my.yearupunited.org"/>
-    <x v="2"/>
+    <s v="idasha lee"/>
     <s v="First visit"/>
     <x v="2"/>
     <s v="Very Satisfied"/>
@@ -1688,16 +2732,16 @@
     <s v="Dissatisfied"/>
     <s v="Food Quality"/>
     <n v="7"/>
-    <x v="2"/>
+    <s v="Birthday Rewards;Coupons or deals (BOGO);Discounts on future purchases;"/>
     <m/>
   </r>
   <r>
-    <x v="3"/>
+    <n v="4"/>
     <d v="2026-10-16T11:13:50"/>
     <d v="2026-10-16T11:14:49"/>
     <d v="1899-12-30T00:00:59"/>
     <s v="tstaana@my.yearupunited.org"/>
-    <x v="3"/>
+    <s v="thania staana"/>
     <s v="Occasionally"/>
     <x v="1"/>
     <s v="Very Satisfied"/>
@@ -1707,16 +2751,16 @@
     <s v="Satisfied"/>
     <s v="Food Quality"/>
     <n v="8"/>
-    <x v="3"/>
+    <s v="Members-only promotions;Coupons or deals (BOGO);Earning points towards free meals;"/>
     <m/>
   </r>
   <r>
-    <x v="4"/>
+    <n v="5"/>
     <d v="2026-10-16T11:13:14"/>
     <d v="2026-10-16T11:15:12"/>
     <d v="1899-12-30T00:01:58"/>
     <s v="alewis3@my.yearupunited.org"/>
-    <x v="4"/>
+    <s v="ajani lewis"/>
     <s v="Once a week"/>
     <x v="1"/>
     <s v="Satisfied"/>
@@ -1726,17 +2770,36 @@
     <s v="Satisfied"/>
     <s v="Food Quality"/>
     <n v="9"/>
-    <x v="4"/>
+    <s v="Earning points towards free meals;Coupons or deals (BOGO);Members-only promotions;"/>
+    <m/>
+  </r>
+  <r>
+    <n v="6"/>
+    <d v="2026-10-16T16:32:30"/>
+    <d v="2026-10-16T16:33:32"/>
+    <d v="1899-12-30T00:01:02"/>
+    <s v="dmendez1@my.yearupunited.org"/>
+    <s v="denae mendez"/>
+    <s v="First visit"/>
+    <x v="3"/>
+    <s v="Satisfied"/>
+    <s v="Very Satisfied"/>
+    <s v="Satisfied"/>
+    <s v="Neutral"/>
+    <s v="Dissatisfied"/>
+    <s v="Pricing"/>
+    <n v="7"/>
+    <s v="Discounts on future purchases;Earning points towards free meals;Birthday Rewards"/>
     <m/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="4">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="5">
   <r>
     <x v="0"/>
-    <n v="1"/>
+    <n v="4"/>
   </r>
   <r>
     <x v="1"/>
@@ -1748,26 +2811,71 @@
   </r>
   <r>
     <x v="3"/>
+    <n v="3"/>
+  </r>
+  <r>
+    <x v="4"/>
     <n v="2"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE9A2D6A-15EA-4DF9-856B-4B075BA6C58C}" name="PivotTable2" cacheId="113" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A17:C34" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2C78AFEC-7409-41FB-83B0-B152E0ED7104}" name="PivotTable2" cacheId="83" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A18:B24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
-    <pivotField compact="0" outline="0" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="6">
         <item x="1"/>
         <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
   </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of How many chose" fld="1" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -1781,39 +2889,22 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{906B1C44-826D-4BB4-B1C5-C573A4D68373}" name="PivotTable1" cacheId="98" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
-  <location ref="A2:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{906B1C44-826D-4BB4-B1C5-C573A4D68373}" name="PivotTable1" cacheId="79" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A2:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
-    <pivotField compact="0" outline="0" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" numFmtId="164" outline="0" showAll="0"/>
     <pivotField compact="0" numFmtId="164" outline="0" showAll="0"/>
     <pivotField compact="0" numFmtId="45" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0">
-      <items count="6">
-        <item x="4"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="4">
+      <items count="5">
         <item x="0"/>
         <item x="2"/>
         <item x="1"/>
+        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -1824,22 +2915,13 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="7"/>
   </rowFields>
-  <rowItems count="4">
+  <rowItems count="5">
     <i>
       <x/>
     </i>
@@ -1848,6 +2930,9 @@
     </i>
     <i>
       <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -1883,8 +2968,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:Q6" totalsRowShown="0">
-  <autoFilter ref="A1:Q6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:Q7" totalsRowShown="0">
+  <autoFilter ref="A1:Q7" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="16">
       <extLst>
@@ -2005,7 +3090,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="N1zOu4HxDE2TEH-Hczbhz5uJQgU128BLhNMOvqdz4P5UOFVNU0Y5VkNPOUZMWk9OTFBKWU0wQUtJNi4u" isFormConnected="1" maxResponseId="5" latestEventMarker="0">
+      <xlmsforms:msForm id="N1zOu4HxDE2TEH-Hczbhz5uJQgU128BLhNMOvqdz4P5UOFVNU0Y5VkNPOUZMWk9OTFBKWU0wQUtJNi4u" isFormConnected="1" maxResponseId="6" latestEventMarker="1">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -2325,13 +3410,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q30"/>
+  <sheetPr>
+    <tabColor rgb="FF0070C0"/>
+  </sheetPr>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
@@ -2341,7 +3429,7 @@
     <col min="11" max="11" width="13.42578125" customWidth="1"/>
     <col min="12" max="12" width="15.7109375" customWidth="1"/>
     <col min="13" max="13" width="16.42578125" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" customWidth="1"/>
     <col min="15" max="15" width="20.42578125" customWidth="1"/>
     <col min="16" max="16" width="23.85546875" customWidth="1"/>
     <col min="17" max="17" width="66.85546875" customWidth="1"/>
@@ -2351,13 +3439,13 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -2404,13 +3492,13 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>46309.869722222225</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>46309.87195601852</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <f t="shared" ref="D2:D6" si="0">C2 - B2</f>
         <v>2.2337962946039625E-3</v>
       </c>
@@ -2458,13 +3546,13 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>46310.601400462961</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>46310.601921296293</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f t="shared" si="0"/>
         <v>5.2083333139307797E-4</v>
       </c>
@@ -2509,13 +3597,13 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>46310.614733796298</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>46310.616493055553</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f t="shared" si="0"/>
         <v>1.7592592557775788E-3</v>
       </c>
@@ -2560,13 +3648,13 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>46311.467939814815</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>46311.468622685185</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <f t="shared" si="0"/>
         <v>6.8287036992842332E-4</v>
       </c>
@@ -2611,13 +3699,13 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>46311.467523148145</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>46311.468888888892</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <f t="shared" si="0"/>
         <v>1.3657407471328042E-3</v>
       </c>
@@ -2658,142 +3746,246 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="4:16">
-      <c r="D22" s="3">
-        <f>AVERAGE(D2:D21)</f>
-        <v>1.3124999997671694E-3</v>
-      </c>
-      <c r="H22">
-        <f>AVERAGE(H2:H21)</f>
-        <v>4</v>
-      </c>
-      <c r="I22" s="4">
-        <f>SUM(COUNTIF(I2:I21,"Satisfied"),COUNTIF(I2:I21,"Very Satisfied"))</f>
+    <row r="7" spans="1:17">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46311.689236111102</v>
+      </c>
+      <c r="C7" s="1">
+        <v>46311.689953703702</v>
+      </c>
+      <c r="D7" s="2">
+        <f>C7 - B7</f>
+        <v>7.1759260026738048E-4</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7">
         <v>3</v>
       </c>
-      <c r="J22" s="4">
-        <f t="shared" ref="J22:M22" si="1">SUM(COUNTIF(J2:J21,"Satisfied"),COUNTIF(J2:J21,"Very Satisfied"))</f>
-        <v>3</v>
-      </c>
-      <c r="K22" s="4">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="L22" s="4">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="M22" s="4">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="O22">
-        <f>AVERAGE(O2:O21)</f>
-        <v>5.8</v>
-      </c>
+      <c r="I7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O7">
+        <v>7</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q7" s="5"/>
     </row>
     <row r="23" spans="4:16">
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
+      <c r="D23" s="2">
+        <f>AVERAGE(D2:D22)</f>
+        <v>1.2133487665172045E-3</v>
+      </c>
+      <c r="H23">
+        <f>AVERAGE(H2:H22)</f>
+        <v>3.8333333333333335</v>
+      </c>
+      <c r="I23" s="3">
+        <f>SUM(COUNTIF(I2:I22,"Satisfied"),COUNTIF(I2:I22,"Very Satisfied"))</f>
+        <v>4</v>
+      </c>
+      <c r="J23" s="3">
+        <f>SUM(COUNTIF(J2:J22,"Satisfied"),COUNTIF(J2:J22,"Very Satisfied"))</f>
+        <v>4</v>
+      </c>
+      <c r="K23" s="3">
+        <f>SUM(COUNTIF(K2:K22,"Satisfied"),COUNTIF(K2:K22,"Very Satisfied"))</f>
+        <v>5</v>
+      </c>
+      <c r="L23" s="3">
+        <f>SUM(COUNTIF(L2:L22,"Satisfied"),COUNTIF(L2:L22,"Very Satisfied"))</f>
+        <v>2</v>
+      </c>
+      <c r="M23" s="3">
+        <f>SUM(COUNTIF(M2:M22,"Satisfied"),COUNTIF(M2:M22,"Very Satisfied"))</f>
+        <v>2</v>
+      </c>
+      <c r="O23">
+        <f>AVERAGE(O2:O22)</f>
+        <v>6</v>
+      </c>
     </row>
-    <row r="24" spans="4:16">
-      <c r="M24" t="s">
-        <v>22</v>
-      </c>
-      <c r="N24">
-        <f>COUNTIF(N2:N21, "Pricing")</f>
-        <v>1</v>
+    <row r="24" spans="4:16" ht="30.75">
+      <c r="F24" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" t="s">
+        <v>47</v>
+      </c>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N24" t="s">
+        <v>49</v>
+      </c>
+      <c r="O24" t="s">
+        <v>50</v>
+      </c>
+      <c r="P24" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="4:16">
+      <c r="F25" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25">
+        <f>COUNTIF(G2:G21,F25)</f>
+        <v>3</v>
+      </c>
       <c r="M25" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="N25">
-        <f>COUNTIF(N2:N21, M25)</f>
+        <f>COUNTIF(N2:N22, "Pricing")</f>
+        <v>2</v>
+      </c>
+      <c r="O25" t="s">
+        <v>52</v>
+      </c>
+      <c r="P25">
+        <f>COUNTIF(P2:P22, "*Earning points towards free meals*")</f>
         <v>4</v>
-      </c>
-      <c r="O25" t="s">
-        <v>43</v>
-      </c>
-      <c r="P25">
-        <f>COUNTIF(P2:P21, "*Earning points towards free meals*")</f>
-        <v>3</v>
       </c>
     </row>
     <row r="26" spans="4:16">
+      <c r="F26" t="s">
+        <v>27</v>
+      </c>
+      <c r="G26">
+        <f>COUNTIF(G2:G21,F26)</f>
+        <v>2</v>
+      </c>
       <c r="M26" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="N26">
-        <f>COUNTIF(N2:N21, M26)</f>
-        <v>0</v>
+        <f>COUNTIF(N2:N22, M26)</f>
+        <v>4</v>
       </c>
       <c r="O26" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="P26">
-        <f>COUNTIF(P2:P21, "*Birthday Rewards*")</f>
-        <v>1</v>
+        <f>COUNTIF(P2:P22, "*Birthday Rewards*")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="4:16">
+      <c r="F27" t="s">
+        <v>54</v>
+      </c>
+      <c r="G27">
+        <f>COUNTIF(G2:G21,F27)</f>
+        <v>0</v>
+      </c>
       <c r="M27" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="N27">
-        <f>COUNTIF(N2:N21, M27)</f>
+        <f>COUNTIF(N2:N22, M27)</f>
         <v>0</v>
       </c>
       <c r="O27" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="P27">
-        <f>COUNTIF(P2:P21, "*Discounts on future purchases*")</f>
-        <v>2</v>
+        <f>COUNTIF(P2:P22, "*Discounts on future purchases*")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="4:16">
+      <c r="F28" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28">
+        <f>COUNTIF(G2:G21,F28)</f>
+        <v>0</v>
+      </c>
       <c r="M28" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="N28">
-        <f>COUNTIF(N2:N21, M28)</f>
+        <f>COUNTIF(N2:N22, M28)</f>
         <v>0</v>
       </c>
       <c r="O28" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="P28">
-        <f>COUNTIF(P2:P21, "*Coupons or deals (BOGO)*")</f>
+        <f>COUNTIF(P2:P22, "*Coupons or deals (BOGO)*")</f>
         <v>3</v>
       </c>
     </row>
     <row r="29" spans="4:16">
+      <c r="F29" t="s">
+        <v>38</v>
+      </c>
+      <c r="G29">
+        <f>COUNTIF(G2:G21,F29)</f>
+        <v>1</v>
+      </c>
       <c r="M29" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="N29">
-        <f>COUNTIF(N2:N21, M29)</f>
+        <f>COUNTIF(N2:N22, M29)</f>
         <v>0</v>
       </c>
       <c r="O29" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="P29">
-        <f>COUNTIF(P2:P21, "*Members-only promotions*")</f>
+        <f>COUNTIF(P2:P22, "*Members-only promotions*")</f>
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="4:16">
       <c r="M30" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="N30">
-        <f>COUNTIF(N2:N21, M30)</f>
+        <f>COUNTIF(N2:N22, M30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="4:16">
+      <c r="M31" t="s">
+        <v>63</v>
+      </c>
+      <c r="N31">
+        <f>COUNTIF(N2:N22, M31)</f>
         <v>0</v>
       </c>
     </row>
@@ -2808,32 +4000,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEA4894-EED4-497B-9B70-C1E6D20F4721}">
-  <dimension ref="A2:C34"/>
+  <sheetPr>
+    <tabColor rgb="FF00B050"/>
+  </sheetPr>
+  <dimension ref="A2:B24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="62.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="82.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.7109375" customWidth="1"/>
+    <col min="4" max="4" width="47.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="82.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="6">
         <v>1</v>
       </c>
     </row>
@@ -2841,7 +4036,7 @@
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="6">
         <v>1</v>
       </c>
     </row>
@@ -2849,107 +4044,81 @@
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="1">
-        <v>5</v>
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6">
+        <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="7"/>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="6">
+        <v>6</v>
+      </c>
     </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="10"/>
+    <row r="18" spans="1:2">
+      <c r="A18" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="10"/>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="6">
+        <v>2</v>
+      </c>
     </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="8"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="10"/>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="6">
+        <v>3</v>
+      </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="8"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="10"/>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" s="6">
+        <v>3</v>
+      </c>
     </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="8"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="10"/>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="6">
+        <v>4</v>
+      </c>
     </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="8"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="10"/>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="6">
+        <v>2</v>
+      </c>
     </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="8"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="10"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="8"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="10"/>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="8"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="10"/>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="8"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="10"/>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="8"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="10"/>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="8"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="10"/>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="8"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="10"/>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="8"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="10"/>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="8"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="10"/>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" s="8"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="10"/>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="13"/>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="6">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>